<commit_message>
docs: fold Endless Mode and the solvability oracle into the submission package
features_list.md/.pdf: added #96 Endless Mode and #97 the solvability
oracle (97 features total), with the SPEC.md "Endless Mode" gap note
updated to say it was closed this session rather than left open.

testing_tasks.md/.pdf: extended Member A's Levels & World row to cover
manually verifying both.

Member_Contributions.md/.pdf/.xlsx: two more task rows for this session's
Endless Mode + solvability oracle implementation and the submission-package
rebuild itself (120 tasks, 223.5 hours total).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submission_documents/Member_Contributions.xlsx
+++ b/submission_documents/Member_Contributions.xlsx
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>214.5</v>
+        <v>223.5</v>
       </c>
     </row>
     <row r="8">
@@ -638,16 +638,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E14" t="n">
-        <v>0.618644</v>
+        <v>0.625</v>
       </c>
       <c r="F14" t="n">
-        <v>134.5</v>
+        <v>143.5</v>
       </c>
       <c r="G14" t="n">
-        <v>0.62704</v>
+        <v>0.642058</v>
       </c>
       <c r="H14" t="n">
         <v>258</v>
@@ -680,13 +680,13 @@
         <v>45</v>
       </c>
       <c r="E15" t="n">
-        <v>0.381356</v>
+        <v>0.375</v>
       </c>
       <c r="F15" t="n">
         <v>80</v>
       </c>
       <c r="G15" t="n">
-        <v>0.37296</v>
+        <v>0.357942</v>
       </c>
       <c r="H15" t="n">
         <v>58</v>
@@ -712,7 +712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4045,23 +4045,79 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>25125084</t>
+          <t>25125083</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Trần Gia Huy</t>
+          <t>Nguyễn Đình Minh Huy</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
+          <t>Implemented Endless Mode (chunked infinite level generation with rising difficulty, distance-based scoring) and a real solvability oracle for MapGenerator, after evaluating (and rejecting the framework of) the abandoned A/mapgen-gan-plan and A/rl-neural-policy side branches for anything worth porting</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>5</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>this session, branch A/feature/endless-mode-and-solvability</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>119</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Rebuilt the submission package: a 97-feature list and per-member manual test checklist grounded in a fresh source-code audit, the Member Contributions spreadsheet (matching the DesignPatternsGroup52 format), and an expanded report (OOP/pattern rationale, two new UML diagrams)</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>4</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>this session, branch A/docs/submission-package-update</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>120</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>25125084</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Trần Gia Huy</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
           <t>Resolved merge conflicts while pulling the latest changes and merged into main</t>
         </is>
       </c>
-      <c r="E120" t="n">
+      <c r="E122" t="n">
         <v>2</v>
       </c>
-      <c r="F120" t="inlineStr">
+      <c r="F122" t="inlineStr">
         <is>
           <t>Git commits 72b13c6, a522007, 75e9cbb</t>
         </is>

</xml_diff>

<commit_message>
docs: generate Member_Contributions from one script, extend to 09-02
Write scripts/build_contributions.py so Member_Contributions.md and
.xlsx are rendered from one in-script task table instead of being
hand-synced (no generator existed before this; the xlsx was written
directly with openpyxl on 2026-08-31). The script also measures Git
commit counts live via `git shortlog -sn` instead of a typed-in number.

Extend the task table from #121 with the 2026-08-31 .. 2026-09-02
sessions (37 new rows, 97.5h, all Member A per the log - no B/ branch
entries appear in this window), for 157 tasks / 321 hours total.
Refreshed commit counts: Nguyen Dinh Minh Huy 417, Tran Gia Huy +
FubuGold (Member B) 61, total 478 (previously 316).
</commit_message>
<xml_diff>
--- a/submission_documents/Member_Contributions.xlsx
+++ b/submission_documents/Member_Contributions.xlsx
@@ -40,6 +40,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDDDDD"/>
+        <bgColor rgb="00DDDDDD"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,13 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -504,7 +502,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>120</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7">
@@ -514,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>223.5</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +522,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>316</v>
+        <v>478</v>
       </c>
     </row>
     <row r="9">
@@ -638,22 +636,22 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>75</v>
+        <v>112</v>
       </c>
       <c r="E14" t="n">
-        <v>0.625</v>
+        <v>0.7133757961783439</v>
       </c>
       <c r="F14" t="n">
-        <v>143.5</v>
+        <v>241</v>
       </c>
       <c r="G14" t="n">
-        <v>0.642058</v>
+        <v>0.7507788161993769</v>
       </c>
       <c r="H14" t="n">
-        <v>258</v>
+        <v>417</v>
       </c>
       <c r="I14" t="n">
-        <v>0.816456</v>
+        <v>0.8723849372384938</v>
       </c>
       <c r="J14" t="n">
         <v>0.5</v>
@@ -680,19 +678,19 @@
         <v>45</v>
       </c>
       <c r="E15" t="n">
-        <v>0.375</v>
+        <v>0.286624203821656</v>
       </c>
       <c r="F15" t="n">
         <v>80</v>
       </c>
       <c r="G15" t="n">
-        <v>0.357942</v>
+        <v>0.2492211838006231</v>
       </c>
       <c r="H15" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I15" t="n">
-        <v>0.183544</v>
+        <v>0.1276150627615063</v>
       </c>
       <c r="J15" t="n">
         <v>0.5</v>
@@ -712,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F122"/>
+  <dimension ref="A1:F159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -724,7 +722,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>A task should be done by only 1-2 students. Duplicate tasks are not recommended
 Each member should work on at least 5 tasks</t>
@@ -732,32 +730,32 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Student ID</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Full name</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Task Description</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Hours</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>Evidence (screenshots of chat messages, of Git commits... proving that you perform and finish the task)</t>
         </is>
@@ -4120,6 +4118,1042 @@
       <c r="F122" t="inlineStr">
         <is>
           <t>Git commits 72b13c6, a522007, 75e9cbb</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>121</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Merged all outstanding work to dev/main and generated the initial submission package (AI Usage Declaration, features list, task division, demo-video placeholder, member contributions, final report) while kicking off the defect-auditing test suite.</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>3</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>see logs/agent_history.log 2026-08-30, branch main</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>122</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Merged the level-completion, endless-mode, and submission-package branches into dev then main and pushed; corrected the AI Usage Declaration's tool attribution (Antigravity vs. Claude Code) per user feedback.</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>1</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>see logs/agent_history.log 2026-08-31 09:45 and 10:00, branch main</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>123</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Replaced the report's ASCII architecture diagram with a real figure, embedded full-depth UML diagrams in the appendix, and rewrote the class-diagram generator to render every attribute/method with UML visibility notation, fixing a brace-init parsing bug along the way.</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>branches A/docs/report-architecture-figure-and-full-uml, A/docs/detailed-uml-full-attributes-methods</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>124</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Ran a three-way SPEC/code/report audit via three parallel subagent passes, producing a 15-defect, 14-task (R1-R14) remediation plan and correcting nine stale claims in the features list and report.</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>4</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>branch A/docs/spec-feature-audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>125</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Small-defect and hygiene batch (R1/R2/R3/R6): fixed SoundManager's level-BGM index mapping, Enemy/Spiny's screen-height despawn bug, and unsurfaced solvability results; deleted the dead AnimationManager class; degraded audio startup gracefully with no device; untracked .member_profile.json and added SPEC's descope addendum.</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>see logs/agent_history.log 2026-08-31 11:48-12:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>126</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Migrated every raw EventBus SubscriptionId to ScopedSubscription across PlayingState/AchievementManager/StatisticsTracker/Camera (R4), and fixed a real static-destruction-order SIGSEGV the migration surfaced.</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>branch A/fix/scoped-subscription-adoption, commit 00c08f8</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>127</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Fixed a P-Switch soft-lock caused by mis-themed sub-level floors, a half-rendered single-column pipe in all three sub-levels, and made the overworld QuestionBlock's sprite reflect its emptied state to match SPEC (R16).</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>3</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>branch A/fix/sublevel-tile-batch, commit cc6a32d</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>128</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Investigated reported 'Bowser never spawns' and 'flag reachable mid-fight' defects (both refuted as already fixed/non-reproducing) and widened Boom Boom's arena from 3.5 to 12.5 tiles of pacing room by removing decorative staircase tiles (R15).</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>branch A/fix/boss-encounter-batch, commit 56c8db7</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>129</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Fixed the end-game audio batch: castle_complete fanfare being clobbered by level_complete on boss levels via a deferred one-shot-music swap; investigated and struck two further audio defects as not reproducible/already fixed (R19).</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>2</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>branch A/fix/endgame-audio-batch, commit de52042</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>130</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Reconciled the SPEC-audit document's defect ledger against shipped code, marking or striking about twenty defects and phases (R1-R19) and documenting four previously mis-recorded playtest defects.</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>1</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>branch A/docs/audit-status-reconciliation, commit cc08fc3</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>131</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Fixed the Star power's missing rainbow-tint visual, the sub-level Piranha Plant's pipe-centering offset, and the fireball-kill flip-death sprite anchor via a shared Entity::drawSprite fix reaching every flip-killable enemy (R17).</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>branch A/fix/player-enemy-visual-batch, commit 4550bfe</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>132</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Eliminated all 28 real dynamic_casts from CollisionResolver/PhysicsEngine via new virtual Entity/Item/Block/Enemy/Character hooks (nine commits, one dispatch family each), adding 26 regression checks and discovering that Release's -DNDEBUG compiled away nearly all existing assert()-based coverage (R5).</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>4</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>branch A/refactor/collision-dispatch, commit 4b87e0d</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>133</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Placed all six previously-unused enemy types (KoopaParatroopa, Boo, BulletBill, Thwomp, ChainChomp, Lakitu) and hidden blocks across the campaign, fixed the secret_finder achievement's wrong trigger condition, and fixed two playtest-found defects in Bullet Bill and Lakitu placement (R9).</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>4</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>branch A/feature/campaign-population-pass, commit 4d6be7e</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>134</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Stripped -DNDEBUG from ctest targets only (fixing vacuously-passing assert-based harnesses), refactored the build to compile app sources once via two CMake OBJECT libraries, and added a mutation-tested guard against tests writing into the real saves/ directory (R11).</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>4</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>branches A/fix/tests-honour-assertions, A/build/object-library, A/fix/hermetic-tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>135</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Wired eight dormant systems into real gameplay: star-power side-touch kills, four unused particle types, surface-dependent footsteps, combo-hit pitch escalation, menu-row navigation SFX, a single-player camera clamp, and debug-console tab-completion (R7).</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>3</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>branch A/feature/wire-dormant-vfx-sfx, commit 7d94fb9</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>136</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Added a keyboard-navigable LOAD GAME menu with a 3-slot picker showing character/level/score/time previews, reusing PlayingState's existing loadFromSlot path (R8).</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>branch A/feature/load-game-menu, commit d6672b7</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>137</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Implemented main-menu Attract Mode (30s idle triggers a bundled demo replay, dismissed by any key), fixing two latent ReplayRecorder playback-pacing/fade-in bugs surfaced by actually watching it run (R10).</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>3</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>branch A/feature/attract-mode, commit 6075c27</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>138</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Ran a full scripted playtest evidence pass across campaign completion, P-Switch/POW/axe, 2P versus death, difficulty modes, key rebinding, and FPS, discovering two new defects: boss destroyed by the respawn-safety sweep, and Load Game always resuming World 1-1 (R12).</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>3</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>branch A/verify/full-playtest-pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>139</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Fixed the boss-survives-respawn defect (D29), Load Game restoring the saved level (D30), and re-implemented a double-exit guard for PlayingState, each with a mutation-tested regression case; merged and independently re-verified into dev (R20).</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>3</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>branch A/fix/remaining-defects-d29-d30-exit, commit 6e4868d</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>140</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Root-caused and fixed a user-reported bug where Bowser fell out of the world through his own bridge/lava floor, since the void-plane check only covered players; added an Entity::onLeftLevel virtual hook.</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>2</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>branch A/fix/boss-falls-out-of-world, commit 95521a8</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>141</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Fixed ten gameplay/visual issues in one pass: castle sprite/position, level-clear music timing, Star invincibility flicker, Piranha Plant centering, fireball flip pivot, Bowser arena verification, bonus-level plateau/castle seating, and Peach's Space-key float.</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>3</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>see logs/agent_history.log 2026-09-01 15:31 and 16:52, branch dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>142</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Fixed sub-level pipe teleports and half-sprite rendering, decoupled the S key from ground-pound (crouch-only), halved Thwomp slam speed with a narrowed detection column, rewrote Chain Chomp's tethered-chase AI, enclosed the 1-3 bridge with walls, and fixed the camera snap on Bowser's defeat.</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>3</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>see logs/agent_history.log 2026-09-01 17:55, branch dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>143</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Wrote the demo-video-requirements checklist; fixed the M-key minimap toggle, a duplicate player-death animation, metal-footstep SFX volume, and further tuned Thwomp slam/recovery speed and its 1-3 placement.</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>see logs/agent_history.log 2026-09-01 23:30, branch dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>144</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>R21 Phase 1 defect batch: fixed twelve release defects in one pass — a duplicate untracked asset tree causing level-data drift, half/warped pipe rendering, spawns embedded in solid tiles, an incomplete castle slab, double-integrated moving platforms, menu text overflow, duplicate achievement toasts, and gated debug ImGui off by default.</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>4</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>branch A/release/defect-batch-r21, commit 171a5b3</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>145</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Merged the R21 batch and completed Phases 2-4: built a real GUI level editor wired to EntityFactory (fixing 24 of 40 silently-broken palette buttons), debug/recording cheats with a void-rescuing Immortal mode, fixed far-chunk procedural entities teleporting back to chunk-local coordinates, an explicit entity-type registry, and Bonus D's dynamic day/night lighting via a real GLSL shader.</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>commit 97fc43a (merge into dev), branch A/release/defect-batch-r21</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>146</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Second user-reported defect wave: fixed warp-pipe hitbox/art and entry-mode rendering, Bowser's fireball stagger triple-counting a single fireball as three hits, Bowser falling into lava, Lakitu dropping a Fire Flower to keep the fight winnable, the 2P camera freezing on the eliminated player instead of following the survivor, and added save-slot choice/delete.</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>commit e97b7da (merge), branch A/fix/versus-camera-and-axes</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>147</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Audited OOP/SOLID adherence and design-pattern fidelity across the codebase (dynamic_cast counts, singleton count, friend-class audit, PDF text-overlap root cause) and authored the phased submission-sweep plan with per-lane dependencies, models, and effort levels.</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>3</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>docs/issues/submission_sweep_plan_2026-09-02.md, branch dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>148</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Ran the submission-sweep Phase 0 baseline: clean rebuild, full ctest/regression run, a live smoke-test launch, and confirmed the LevelSolvability fix, with no code changes.</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>1</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>see logs/agent_history.log 2026-09-02 18:58, branch dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>149</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Wrote the W11, W12, and W13 weekly reports from git log and agent-history evidence, including tracing the World 1-3 mid-frame entity-spawn crash's root cause for W11.</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>3</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>branches A/docs/weekly-w11, A/docs/weekly-w12-w13</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>150</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Archived 20+ stale root/docs artifacts to docs/archive/, untracked stale saves/PDFs/zips, then reverted an AGENTS.md edit that had landed inside AgentHub's generated block and routed the rule change upstream instead.</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>2</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>branch A/chore/archive-2026-09-02, commit 9b83c9a</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>151</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Extended the AI Usage Declaration to cover the full R1-R21 remediation plan, then corrected its date range and removed an unverifiable test-count claim per review.</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>1</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>branch A/docs/ai-declaration, commit 96560bd</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>152</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Captured fresh gameplay screenshots and composited three YouTube thumbnail candidates, then narrowed to one final crop-and-zoom version after review found Mario illegibly small at native resolution.</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>branch A/docs/video-thumbnail</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>153</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Fixed the report PDF's overlapping-table-text defect with content-aware column sizing, added a build.sh Overfull-hbox guard, and split two illegible full-detail UML pages into landscape multi-page spreads.</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>branch A/docs/report-layout, commit 0f3e5ea</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>154</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Fixed the level editor's F5 playtest routing to Game Over/main menu instead of popping back to the editor on death, with a mutation-tested regression case.</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>branch A/fix/editor-playtest-gameover, commit 2bd2f80</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>155</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Fixed MapGenerator's procedurally-generated vault exit pipe defaulting to the wrong entry mode; investigated the reported 'unreachable third Hard-mode axe' and found it does not reproduce, shipping a protective regression guard instead of an unjustified data edit.</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>branch A/fix/hard-axe-and-vault-pipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>156</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Added a camera-distance gate on Endless Mode's ever-growing entity list, added ImGui sliders for the dynamic-lighting tunables, and deleted the dead UiRenderer::wrapText function.</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>2</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>branch A/fix/endless-gate-lighting-sliders-wraptext, commit 0fe7138</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>157</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>25125083</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Nguyễn Đình Minh Huy</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Fixed MovingPlatform never advancing its own animation, flipped Spiny's default to spawn as an unhatched egg matching SPEC, and added a hardened post-condition regression test after review found the original test too weak.</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>2</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>branch A/fix/moving-platform-and-spiny-egg, commit cf195cb</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: stamp Member_Contributions' git counts with the commit and date measured
Live git counts are correct but timeless without this: a grader could
not tell when "480 commits" was true, and it was already stale by the
time of the prior commit (417 -> 419 just from those two commits
landing). Add get_git_sha() (same subprocess pattern as
count_git_commits) and print "Git commit counts measured at <sha> on
<date>." near the Summary in both editions. Do not freeze the counts -
measuring live is correct; the stamp is what makes a measurement honest
rather than presented as timeless.
</commit_message>
<xml_diff>
--- a/submission_documents/Member_Contributions.xlsx
+++ b/submission_documents/Member_Contributions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="9">
@@ -548,154 +548,161 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Do not edit the grey cells. TAs will enter the score of all PAs in the project score and get the individual scores. Students can enter an estimated project score to see how percentages affects your scores</t>
+          <t>Git commit counts measured at 30f00d8 on 2026-09-02.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Do not edit the grey cells. TAs will enter the score of all PAs in the project score and get the individual scores. Students can enter an estimated project score to see how percentages affects your scores</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Use columns Tasks - Percent, Task Hours - Percent, Git - Percent as references for column Percent</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Student ID</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Full name</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Tasks</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Tasks - Percent</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Task Hours</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Task Hours - Percent</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Git Commits</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Git - Percent</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Percent</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Score - Student</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Score - TA</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>25125083</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Nguyễn Đình Minh Huy</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>112</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0.7133757961783439</v>
-      </c>
-      <c r="F14" t="n">
-        <v>241</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.7507788161993769</v>
-      </c>
-      <c r="H14" t="n">
-        <v>417</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0.8723849372384938</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K14" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>25125084</t>
+          <t>25125083</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Trần Gia Huy</t>
+          <t>Nguyễn Đình Minh Huy</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>45</v>
+        <v>112</v>
       </c>
       <c r="E15" t="n">
-        <v>0.286624203821656</v>
+        <v>0.7133757961783439</v>
       </c>
       <c r="F15" t="n">
-        <v>80</v>
+        <v>241</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2492211838006231</v>
+        <v>0.7507788161993769</v>
       </c>
       <c r="H15" t="n">
-        <v>61</v>
+        <v>419</v>
       </c>
       <c r="I15" t="n">
-        <v>0.1276150627615063</v>
+        <v>0.8729166666666667</v>
       </c>
       <c r="J15" t="n">
         <v>0.5</v>
       </c>
       <c r="K15" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>25125084</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Trần Gia Huy</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>45</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.286624203821656</v>
+      </c>
+      <c r="F16" t="n">
+        <v>80</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.2492211838006231</v>
+      </c>
+      <c r="H16" t="n">
+        <v>61</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.1270833333333333</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K16" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>